<commit_message>
add new menu /cetak
</commit_message>
<xml_diff>
--- a/data/IDP.xlsx
+++ b/data/IDP.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\porto\idp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD43EDE-3F9E-4508-A6C8-873A07C643AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD05F8D-8B74-4CCD-9246-EC6BAEAB2853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7BB28634-8F4E-428D-A0BE-B951B8E62A06}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7BB28634-8F4E-428D-A0BE-B951B8E62A06}"/>
   </bookViews>
   <sheets>
     <sheet name="Teknis" sheetId="1" r:id="rId1"/>
-    <sheet name="Manajerial" sheetId="2" r:id="rId2"/>
-    <sheet name="Sosial Kultural" sheetId="3" r:id="rId3"/>
+    <sheet name="TeknisKasi" sheetId="4" r:id="rId2"/>
+    <sheet name="Manajerial" sheetId="2" r:id="rId3"/>
+    <sheet name="Sosial Kultural" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="95">
   <si>
     <t>Nomenklatur</t>
   </si>
@@ -302,6 +303,69 @@
   </si>
   <si>
     <t>Account Representative</t>
+  </si>
+  <si>
+    <t>Kantor</t>
+  </si>
+  <si>
+    <t>KANTOR WILAYAH DIREKTORAT JENDERAL PAJAK SELAIN KANTOR WILAYAH WAJIB PAJAK BESAR DAN KANTOR WILAYAH JAKARTA KHUSUS</t>
+  </si>
+  <si>
+    <t>10.Advokasi
+Kebijakan
+Perpajakan</t>
+  </si>
+  <si>
+    <t>Kepala Subbagian Kepegawaian</t>
+  </si>
+  <si>
+    <t>11.Manajemen
+Sumber Daya
+Manusia
+Aparatur Sipil
+Negara</t>
+  </si>
+  <si>
+    <t>2.1. Menyusun
+program/rencana kerja,
+materi, instrumen/alat
+bantu, dan/atau
+kelengkapan pelaksanaan
+advokasi kebijakan;
+2.2. Mengidentifikasi aspek
+monitoring dan evaluasi
+atas kegiatan advokasi serta
+kebutuhan tindak lanjut
+advokasi yang spesifik dan
+intensif sesuai lingkup
+tugas;
+2.3. Melakukan analisis bahan
+dalam rangka penyusunan
+kebijakan operasional
+berdasarkan konsep
+kebijakan nasional sesuai
+lingkup tugas.</t>
+  </si>
+  <si>
+    <t>3.1. Mampu melakukan analisi
+terhadap hasil pengolahan
+data kepegawaian;
+(pemetaan pegawai, mutasi,
+promosi, dll);
+3.2. Mampu menyusun
+instrumen dan/atau
+pelaksanaan tahapan dalam
+manajemen SDM
+(perencanaan kebutuhan,
+rekruitmen, analisis
+jabatan, analisis beban
+kerja, evaluasi jabatan,
+perencanaan kinerja,
+standar kompetensi,
+perencanaan
+pengembangan kompetensi,
+pemeringkatan jabatan/job
+grading, dll);</t>
   </si>
 </sst>
 </file>
@@ -1082,6 +1146,67 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA89B6DE-E7FE-4485-ACE7-77E820D6C9F8}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA03166F-B64E-4321-9F54-C8EE3B03B108}">
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1283,7 +1408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E87BED-841E-4804-BE86-914FE8AFA517}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>